<commit_message>
Add expense Hebrew descriptions
</commit_message>
<xml_diff>
--- a/finance/expenses.xlsx
+++ b/finance/expenses.xlsx
@@ -75,12 +75,13 @@
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="34" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="34" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -104,32 +105,37 @@
           <t>Описание</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Описание, иврит</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t>Сумма, ILS</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t>НДС, ILS</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t>Способ оплаты</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t>Документ</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t>Статус проверки</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="1">
         <is>
           <t>Комментарий</t>
         </is>
@@ -156,26 +162,81 @@
           <t>Стрижка кустов; оплата за июнь 2026</t>
         </is>
       </c>
-      <c r="E2" s="0">
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t>גיזום שיחים; תשלום עבור יוני 2026</t>
+        </is>
+      </c>
+      <c r="F2" s="0">
         <v>1030</v>
       </c>
-      <c r="G2" t="inlineStr" s="0">
+      <c r="H2" t="inlineStr" s="0">
         <is>
           <t>не указано</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr" s="0">
+      <c r="J2" t="inlineStr" s="0">
         <is>
           <t>требует проверки</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr" s="0">
+      <c r="K2" t="inlineStr" s="0">
         <is>
           <t>Квитанция не получена; забрать и напомнить садовнику</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Сантехника</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>מ.ח. תיקונים</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Квартира 6 — ремонт канализации / устранение засора</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>דירה 6 — תיקון ביוב / פתיחת סתימה</t>
+        </is>
+      </c>
+      <c r="F3" s="0">
+        <v>750</v>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="I3" s="0" t="inlineStr">
+        <is>
+          <t>documents/receipts/2026-06-25-apartment-6-sewer-repair-750-ils.pdf</t>
+        </is>
+      </c>
+      <c r="J3" s="0" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="K3" s="0" t="inlineStr">
+        <is>
+          <t>Квитанция №0298; дата на квитанции 25.6.26; сумма 750 ₪</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J2"/>
+  <autoFilter ref="A1:K3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add June expenses report and apartment 8 signature
</commit_message>
<xml_diff>
--- a/finance/expenses.xlsx
+++ b/finance/expenses.xlsx
@@ -154,17 +154,17 @@
       </c>
       <c r="C2" t="inlineStr" s="0">
         <is>
-          <t>Садовник — יוסף גנן</t>
+          <t>פסגת הגנים</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="0">
         <is>
-          <t>Стрижка кустов; оплата за июнь 2026</t>
+          <t>Уход за садом; оплата за июнь 2026</t>
         </is>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
-          <t>גיזום שיחים; תשלום עבור יוני 2026</t>
+          <t>תחזוקת גינה; תשלום עבור יוני 2026</t>
         </is>
       </c>
       <c r="F2" s="0">
@@ -175,14 +175,19 @@
           <t>не указано</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr" s="0">
+        <is>
+          <t>documents/receipts/2026-07-01-gardener-june-2026-1030-ils.pdf</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr" s="0">
         <is>
-          <t>требует проверки</t>
+          <t>подтверждено</t>
         </is>
       </c>
       <c r="K2" t="inlineStr" s="0">
         <is>
-          <t>Квитанция не получена; забрать и напомнить садовнику</t>
+          <t>חשבונית מס/קבלה №030 от 2026-07-01; сумма 1030 ₪</t>
         </is>
       </c>
     </row>

</xml_diff>